<commit_message>
Add script to create manual test cases for document conversion, PDF editing, and image processing
</commit_message>
<xml_diff>
--- a/Manual Test Cases for Option 2.xlsx
+++ b/Manual Test Cases for Option 2.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Manual Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,12 +421,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,15 +479,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Valid DOCX file</t>
+          <t>Valid DOCX file upload</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Successfully converts DOCX to PDF</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>File is converted to PDF format successfully</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -495,7 +499,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Supported valid file format</t>
+          <t>Valid file provided</t>
         </is>
       </c>
     </row>
@@ -517,10 +521,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Error message indicating invalid or corrupted file</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>UI shows error message 'Invalid file'</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -528,7 +536,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>File format validation works</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -545,15 +553,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Unsupported EXE file</t>
+          <t>DOCX file exceeding 50MB size limit</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Error message indicating wrong or unsupported file format</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>UI shows error message 'File too large'</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -561,7 +573,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Strict format extension restrictions</t>
+          <t>Limit is 50MB</t>
         </is>
       </c>
     </row>
@@ -578,15 +590,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Valid PDF and add text</t>
+          <t>Add text annotation to PDF</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Text is added and PDF saves successfully</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Text appears correctly on the PDF canvas</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -594,7 +610,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Normal operation conditions met</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -611,15 +627,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Password-protected PDF</t>
+          <t>Upload password-protected PDF</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Prompt to unlock or clear error message</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Prompt asking for password appears rather than crashing</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -627,7 +647,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Security enforcement handles encryption</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -644,15 +664,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0 byte PDF file</t>
+          <t>Save edits on 0-page empty PDF</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Error message for empty file</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>UI displays error 'Empty document cannot be edited'</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -660,7 +684,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Empty file handling</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -677,15 +701,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Valid JPG, 800x600 size inputs</t>
+          <t>Enter valid dimensions 800x600 px</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Image resized to exactly 800x600</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>Image is resized exactly to 800x600 px rendering clearly</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -693,7 +721,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Valid numeric dimensions accepted</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -710,15 +738,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Width input: -100</t>
+          <t>Enter negative width (e.g., -100) in input</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Validation error requiring positive values</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+          <t>Input field rejects value or shows validation error</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -726,7 +758,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Input boundary constraints</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -743,15 +775,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dimension field with alphabet 'abc'</t>
+          <t>Enter alphabet characters 'abc' in height</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Validation error or ignored input</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>Input field prevents typing letters</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -759,7 +795,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Data type validation on numeric field</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -771,20 +807,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cropping</t>
+          <t>Image resizing</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Valid crop area selection box</t>
+          <t>Select 50% scale from dropdown</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Image cropped strictly to selected area</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>Image scales down to exactly half its original size properly</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -792,7 +832,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Standard behaviour works</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -804,20 +844,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cropping</t>
+          <t>Image resizing</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Crop area outside image boundaries</t>
+          <t>Enter an excessive scale of 5000%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cannot select outside bounds / Snap to edge</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>Validation error showing 'Scale must be under 1000%' in UI</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -825,14 +869,14 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>UI enforces spatial boundaries</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Neg_0008</t>
+          <t>Pos_0005</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -842,15 +886,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0x0 area selection</t>
+          <t>Draw crop box entirely inside image and apply</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Submit disabled or error prompt</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>Image is cropped precisely to the selected region on UI</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -858,32 +906,36 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Minimum crop dimensions configured</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Pos_0005</t>
+          <t>Neg_0008</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Cropping</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Valid 5MB PNG file</t>
+          <t>Drag crop box partially outside image bounds</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Output file size strictly less than 5MB</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>Crop box is properly restricted to image edges</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -891,7 +943,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Compression algorithm runs properly</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -903,20 +955,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Cropping</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0 byte image file</t>
+          <t>Set crop dimensions to 0x0 via handles</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Error message for invalid/empty image payload</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Crop action is disabled or shows error message</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -924,32 +980,36 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Empty file validation triggers</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Neg_0010</t>
+          <t>Pos_0006</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Cropping</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Image exceeding maximum allowed system size (e.g., 5GB)</t>
+          <t>Select 1:1 aspect ratio constraint and drag</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Error stating file too large</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Crop box maintains a perfect square shape during drag</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -957,32 +1017,36 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Server resource limits checked</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pos_0006</t>
+          <t>Neg_0010</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Image format conversion</t>
+          <t>Cropping</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Valid PNG file, target 'JPG' chosen</t>
+          <t>Input negative crop coordinates manually</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Image securely downloaded as valid JPG</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Warning tooltip that coordinates must be positive</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -990,32 +1054,36 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Format library handles convert</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Neg_0011</t>
+          <t>Pos_0007</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Image format conversion</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>No target format selected</t>
+          <t>Upload JPG and select 'High Compression'</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Conversion disabled, warning to select format</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>File size metric drops, visual stays acceptable on display</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1023,32 +1091,36 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Mandatory field check active</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Neg_0012</t>
+          <t>Neg_0011</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Image format conversion</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fake image (txt file manually renamed to .png)</t>
+          <t>Upload a non-image file (.txt)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Error reading or parsing image file</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>UI rejects upload promptly with 'Invalid image format' error</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1056,32 +1128,36 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>File MIME type strict check</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pos_0007</t>
+          <t>Neg_0012</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Meme generation</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Valid text on top and bottom</t>
+          <t>Select 0% (or empty) quality slider</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Meme generated with appropriate text overlay</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>Slider snaps to minimum 1% or shows validation warning</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1089,7 +1165,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Text overlay functional</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1101,20 +1177,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Meme generation</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Extremely long text string (10,000 chars)</t>
+          <t>Upload an already highly compressed 1KB image</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Text truncated or length limit error displayed</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>Notifies user 'File is already maximally compressed'</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1122,32 +1202,36 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Max character limits limit size</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Neg_0014</t>
+          <t>Pos_0008</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Meme generation</t>
+          <t>Image format conversion</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Unsupported binary or zalgo characters</t>
+          <t>Upload PNG and convert to JPG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Characters stripped safely or error returned</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t>Converted file downloads as valid JPG</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1155,32 +1239,36 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Safe encoding validation</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pos_0008</t>
+          <t>Neg_0014</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Color picker</t>
+          <t>Image format conversion</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Click valid pixel within image bounds</t>
+          <t>Upload unsupported format (.xyz)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Correct HEX code displayed instantly</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+          <t>Error message 'Unsupported file format' shown on UI</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1188,7 +1276,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Color extraction parses correct RGBA</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1200,20 +1288,24 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Color picker</t>
+          <t>Image format conversion</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Click outside image on webpage background</t>
+          <t>Convert animated GIF to PNG</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>No color picked / Picker ignores background</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
+          <t>User is warned that animation will be lost on format change</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1221,32 +1313,36 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Canvas bounds checking works</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Neg_0016</t>
+          <t>Pos_0009</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Color picker</t>
+          <t>Meme generation</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Picker action triggered while image is still loading</t>
+          <t>Enter top and bottom text on image template</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Picker disabled or shows loading cursor</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>Text is overlaid properly with white font and black stroke</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1254,32 +1350,36 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Async DOM state handling</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Pos_0009</t>
+          <t>Neg_0016</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Image rotation</t>
+          <t>Meme generation</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Click rotate 90 degrees right</t>
+          <t>Enter exceptionally long text string</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Image appears properly rotated 90 deg</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>Text auto-scales down or wraps without breaking UI layout</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1287,7 +1387,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Transform function applies properly</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1299,20 +1399,24 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Image rotation</t>
+          <t>Meme generation</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Manual angle input 'XYZ'</t>
+          <t>Enter purely blank spaces in text inputs</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Validation error asking for integer</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
+          <t>No text rendered, or validation 'Text cannot be empty'</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1320,32 +1424,36 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Input data type validation</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Neg_0018</t>
+          <t>Pos_0010</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Image rotation</t>
+          <t>Color picker</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Corrupted image uploaded before clicking rotate</t>
+          <t>Click on a solid red area in the image</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>General error loading image initially</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>Color picker correctly displays hex code #FF0000</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1353,32 +1461,36 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Prerequisite dependencies evaluated</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pos_0010</t>
+          <t>Neg_0018</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Image flipping</t>
+          <t>Color picker</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Click flip horizontally</t>
+          <t>Use color picker outside the image area bounds</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Image natively mirrored horizontally</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
+          <t>Action is safely ignored; no color picked</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1386,7 +1498,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Transform CSS applies cleanly</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1398,20 +1510,24 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Image flipping</t>
+          <t>Color picker</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Rapid consecutive spam clicks (10+ times) on flip</t>
+          <t>Click on fully transparent PNG pixel</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>System debounces without browser crash</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
+          <t>Displays transparent code or warns 'No color detected'</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1419,32 +1535,36 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Debounce and queue rate limiting</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Neg_0020</t>
+          <t>Pos_0011</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Image flipping</t>
+          <t>Image rotation</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Flip action on already removed image</t>
+          <t>Click 'Rotate 90° Right' button once</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Error message or UI element resets</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
+          <t>Image rotates exactly 90 degrees clockwise</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1452,32 +1572,36 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>State validity and synchronization</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pos_0011</t>
+          <t>Neg_0020</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Document conversion</t>
+          <t>Image rotation</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Multi-page PDF to DOCX conversion</t>
+          <t>Input '90.5' in custom angle field</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>All pages converted seamlessly into single Doc</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
+          <t>Input field safely rejects decimal values</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1485,7 +1609,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Pagination handlers complete</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1497,20 +1621,24 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Document conversion</t>
+          <t>Image rotation</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Disconnect internet during ongoing conversion</t>
+          <t>Input angle exceeding maximum (e.g. 99999)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Graceful network failure warning message</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+          <t>Angle is neatly rounded modulo 360</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1518,7 +1646,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Frontend network connectivity error handling</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1530,20 +1658,24 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PDF editing</t>
+          <t>Image flipping</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Draw visible rectangle and annotation on page</t>
+          <t>Click 'Flip Horizontal' button</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Shapes and text saved correctly on output PDF</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
+          <t>Image visuals mirror correctly horizontally immediately</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1551,7 +1683,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Draw annotation feature robust</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -1563,20 +1695,24 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PDF editing</t>
+          <t>Image flipping</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Try to delete all pages in a PDF document</t>
+          <t>Click flip buttons before uploading an image</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Warning message or prevent deletion of last page</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
+          <t>Buttons appear disabled, greyed out, or unclickable</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1584,32 +1720,36 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Minimum 1 page baseline rule in PDF spec</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Pos_0013</t>
+          <t>Neg_0023</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Image resizing</t>
+          <t>Image flipping</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>'Keep aspect ratio' checked, edit width</t>
+          <t>Rapid double-click on vertical flip</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Height automatically recalculates appropriately</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
+          <t>UI does not freeze and evaluates both flips natively</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1617,32 +1757,36 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Aspect ratio math executes immediately</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Neg_0023</t>
+          <t>Pos_0013</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Image resizing</t>
+          <t>Image flipping</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Resize to arbitrary massive value (99,999,999 pixels)</t>
+          <t>Click 'Flip Vertical' button on a 1x1 image</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Application error indicating limit threshold reached</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
+          <t>UI updates normally handling extreme bounds correctly</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>Not Executed</t>
@@ -1650,7 +1794,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Sanity scaling limits enforce security against mem abuse</t>
+          <t>NA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add script to generate beautifully formatted Excel file for manual test cases
</commit_message>
<xml_diff>
--- a/Manual Test Cases for Option 2.xlsx
+++ b/Manual Test Cases for Option 2.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sample Template for Option 2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Manual Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,10 +435,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
@@ -498,7 +498,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>System should convert file to PDF format successfully</t>
+          <t>UI shows success state and provides PDF download link</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Valid file provided</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -530,12 +530,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Upload corrupted DOCX file</t>
+          <t>Upload unsupported file format (.txt)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>System should reject file and show 'Invalid file' error</t>
+          <t>UI displays 'Invalid file format' error message</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -567,12 +567,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Upload DOCX file exceeding 50MB limit</t>
+          <t>Drag and drop multiple files when only one is allowed</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>System should show 'File too large' error message</t>
+          <t>UI warns that only one file is permitted at a time</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Limit is 50MB</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -604,12 +604,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Add text annotation to an uploaded PDF</t>
+          <t>Add text annotation tool to canvas</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Text should appear correctly on the PDF canvas</t>
+          <t>Text renders correctly on the PDF preview canvas</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -641,12 +641,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Upload password-protected PDF</t>
+          <t>Apply text annotation completely outside PDF canvas bounds</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>System should prompt for password and not crash</t>
+          <t>Text is clipped or restricted to the canvas boundaries</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -678,12 +678,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Attempt to save edits on 0-page empty PDF</t>
+          <t>Click save changes without making any edits</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>System should display error 'Empty document cannot be edited'</t>
+          <t>Save button is disabled or notifies user of no changes</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -715,12 +715,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Enter valid dimensions 800x600 px</t>
+          <t>Specify exactly 800x600 px dimensions</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Image should resize exactly to 800x600 px rendering clearly</t>
+          <t>Image preview correctly scales to the new dimensions</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -752,12 +752,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Enter negative width (e.g., -100) in input</t>
+          <t>Enter negative number (-50) in height field</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Input field should reject value or show validation error</t>
+          <t>Input field rejects negative input or shows validation</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -789,12 +789,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Enter alphabet characters 'abc' in height</t>
+          <t>Type alphabetic characters ('abc') in width</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Input field should prevent typing letters</t>
+          <t>Letters are ignored by the numeric input field</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -826,12 +826,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Select 50% scale from dropdown</t>
+          <t>Check 'Maintain Aspect Ratio' and change width</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Image should scale down to exactly half its original size</t>
+          <t>Height automatically calculates and updates proportionately</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -853,22 +853,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Neg_0007</t>
+          <t>Pos_0005</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Image resizing</t>
+          <t>Cropping</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Enter an excessive scale of 5000%</t>
+          <t>Draw crop box and click apply crop</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>System should show validation error 'Scale must be under 1000%'</t>
+          <t>Image bounds visually update to the selected crop area</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -890,7 +890,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Pos_0005</t>
+          <t>Neg_0007</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Draw crop box inside image and click apply</t>
+          <t>Drag crop box partially outside image preview</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Image should be cropped precisely to the selected region</t>
+          <t>Crop box perfectly snaps and restricts to preview edges</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -937,12 +937,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Drag crop box partially outside image bounds</t>
+          <t>Drag crop handles so width is practically 0</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>System should properly restrict crop box to image edges</t>
+          <t>Handles restricts to a minimum visual crop size (e.g. 1x1)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Set crop dimensions to 0x0 via handles</t>
+          <t>Double click crop button without drawing crop box</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Crop action should be disabled or show error message</t>
+          <t>Validation message prompts user to draw a box first</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1006,17 +1006,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Cropping</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Select 1:1 aspect ratio constraint and drag</t>
+          <t>Move compression slider to 50% and apply</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Crop box should maintain a perfect square shape</t>
+          <t>Preview visually updates to reflect compressed image</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1043,17 +1043,17 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Cropping</t>
+          <t>Compression</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Input negative crop coordinates manually</t>
+          <t>Enter 150% in manual compression text box</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Warning tooltip should state coordinates must be positive</t>
+          <t>Value auto-corrects to maximum 100% or shows warning</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Pos_0007</t>
+          <t>Neg_0011</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1085,12 +1085,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Upload JPG and select 'High Compression'</t>
+          <t>Submit compression with slider at 0%</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>File size metric should drop while visual stays acceptable</t>
+          <t>Value snaps to minimum 1% without throwing console errors</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1112,7 +1112,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Neg_0011</t>
+          <t>Pos_0007</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Upload a non-image file (.txt)</t>
+          <t>Click reset after applying compression</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>System should reject upload with 'Invalid image format' error</t>
+          <t>Preview perfectly reverts to original uncompressed image</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1149,22 +1149,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Neg_0012</t>
+          <t>Pos_0008</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Image format conversion</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Select 0% (or empty) quality slider</t>
+          <t>Select Convert PNG to JPG and click convert</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Slider should snap to minimum 1% or show validation warning</t>
+          <t>UI provides a JPG conversion success download button</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1186,22 +1186,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Neg_0013</t>
+          <t>Neg_0012</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Compression</t>
+          <t>Image format conversion</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Upload an already highly compressed 1KB image</t>
+          <t>Attempt to convert JPG to JPG</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>System should notify user 'File is already maximally compressed'</t>
+          <t>Format option is disabled or shows already in format alert</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1223,7 +1223,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Pos_0008</t>
+          <t>Neg_0013</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1233,12 +1233,12 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Upload PNG and convert to JPG</t>
+          <t>Leave target format dropdown completely empty</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Converted file should download as a valid JPG</t>
+          <t>Validation states 'Please select a target format'</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1260,22 +1260,22 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Neg_0014</t>
+          <t>Pos_0009</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Image format conversion</t>
+          <t>Meme generation</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Upload unsupported format (.xyz)</t>
+          <t>Enter Top and Bottom text</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Error message 'Unsupported file format' should be shown</t>
+          <t>Text visibly overlays the image preview with standard meme font</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1297,22 +1297,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Neg_0015</t>
+          <t>Neg_0014</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Image format conversion</t>
+          <t>Meme generation</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Convert animated GIF to PNG</t>
+          <t>Submit meme generation without uploading image</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>User should be warned that animation will be lost</t>
+          <t>Validation prompts 'Please upload an image first'</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1334,7 +1334,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Pos_0009</t>
+          <t>Neg_0015</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1344,12 +1344,12 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Upload valid image and add meme text</t>
+          <t>Type text far exceeding typical character length</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Meme preview should display with text</t>
+          <t>Text scales down or wraps instead of overflowing the image</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1381,12 +1381,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Generate meme without uploading image</t>
+          <t>Submit with both inputs containing only spaces</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>System should prevent meme generation</t>
+          <t>Validation flags 'Text cannot be empty'</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1401,29 +1401,29 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Meme generation requires image input</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Neg_0017</t>
+          <t>Pos_0010</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Meme generation</t>
+          <t>Color picker</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Enter very long meme text</t>
+          <t>Click specific specific red pixel on image</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>System should handle text properly</t>
+          <t>HEX code field updates matching the clicked color</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1445,7 +1445,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Pos_0010</t>
+          <t>Neg_0017</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Select a color using the picker and copy HEX/RGB value</t>
+          <t>Click empty background outside the image</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Selected color should update correctly and copied value should match the selected color</t>
+          <t>Color picker ignores click and HEX field remains unchanged</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1492,12 +1492,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Click 'Copy' button without selecting or changing any color</t>
+          <t>Manually type 'ZZZZZZ' into HEX input field</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>System should copy the default selected color value correctly or notify the user if no color is selected</t>
+          <t>Rejects invalid HEX string and reverts to last valid color</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1519,22 +1519,22 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Neg_0019</t>
+          <t>Pos_0011</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Color picker</t>
+          <t>Image rotation</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Try to manually enter invalid color values OR interact randomly with picker</t>
+          <t>Click 'Rotate Right' button once</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>System should restrict invalid inputs or maintain valid color range</t>
+          <t>Image visually rotates exactly 90 degrees clockwise</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1556,7 +1556,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Pos_0011</t>
+          <t>Neg_0019</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Upload valid image and rotate</t>
+          <t>Input special characters into custom angle field</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Image should rotate correctly</t>
+          <t>Input safely ignores all non-numeric characters</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1603,12 +1603,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Click rotate without uploading image</t>
+          <t>Interact with rotate controls before uploading image</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>System should prevent rotation</t>
+          <t>Controls dynamically appear greyed out or disabled</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1623,14 +1623,14 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Image is required before rotation</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Neg_0021</t>
+          <t>Pos_0012</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1640,12 +1640,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Upload unsupported .txt file</t>
+          <t>Click 'Rotate Left' exactly 4 times in a row</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>System should reject invalid file</t>
+          <t>Image visually returns identically to its original unrotated state</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -1660,14 +1660,14 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Rotation works only for images</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Pos_0012</t>
+          <t>Pos_0013</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1677,12 +1677,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Upload valid image and flip</t>
+          <t>Click 'Flip Horizontal' toggle</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Image should flip correctly</t>
+          <t>Image preview correctly mirrors instantly along the Y-axis</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1704,7 +1704,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Neg_0022</t>
+          <t>Neg_0021</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1714,12 +1714,12 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Click flip without uploading image</t>
+          <t>Click flip buttons continuously with no image</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>System should prevent flipping</t>
+          <t>UI produces no errors and leaves the buttons inactive</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -1734,14 +1734,14 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Image is required before flipping</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Neg_0023</t>
+          <t>Neg_0022</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Rapid double-click on vertical flip</t>
+          <t>Extremely rapid multi-clicks on Flip Vertical button</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>System should handle rapid flips natively without freezing</t>
+          <t>UI queue handles flips sequentially without browser freezing</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -1778,7 +1778,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Pos_0013</t>
+          <t>Neg_0023</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1788,12 +1788,12 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Click 'Flip Vertical' button on a 1x1 image</t>
+          <t>Click and drag the flip button instead of pressing</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>UI should update normally handling extreme bounds correctly</t>
+          <t>Button produces standard HTML drag behavior but no flip trigger</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add script to format Excel file for manual test cases
</commit_message>
<xml_diff>
--- a/Manual Test Cases for Option 2.xlsx
+++ b/Manual Test Cases for Option 2.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Manual Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,1371 +433,1380 @@
   </sheetPr>
   <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TC ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Application Feature Tested</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Expected output</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Actual output</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Assumption for Expected Output</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Pos_0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Upload valid DOCX file and click convert</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>File successfully converts to PDF and download link appears</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Neg_0001</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Upload an unsupported HTML file</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>System rejects the file and shows an 'Invalid format' message</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Neg_0002</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Click convert without uploading any file</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>System shows an error message prompting to upload a file first</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Pos_0002</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Add a text box to the PDF and type 'Test'</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Text box appears on the PDF and displays 'Test'</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Neg_0003</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Try to save a PDF without making any changes</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>System should indicate that no changes were made to save</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Neg_0004</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Place a text box outside the PDF page canvas</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Text box is constrained to the PDF page boundaries</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Pos_0003</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Enter width 500 and height 500</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Image preview resizes to the specified 500x500 dimensions</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Pos_0004</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Select 'Maintain aspect ratio' and change width</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Height automatically updates to maintain the original aspect ratio</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Neg_0005</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Enter alphabetical characters ('abc') in the width field</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Input is rejected, and only numeric values are allowed</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Neg_0006</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Enter a negative value (-100) for height</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>System displays a validation error for negative dimensions</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Pos_0005</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Draw a valid crop rectangle and click apply</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Image is cropped exactly to the defined rectangle</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Pos_0006</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Select predefined 1:1 format and apply crop</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Crop boundaries lock into a perfect square</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Neg_0007</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Attempt to drag crop handles completely off the image</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Crop handles automatically snap back to the image edges</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Neg_0008</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Click apply crop without drawing any crop box</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>System warns the user to select an area to crop first</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Pos_0007</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Adjust compression slider to 30%</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Preview updates and estimated file size is appropriately reduced</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Pos_0008</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Click reset after compressing</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Image preview completely reverts to original uncompressed quality</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Neg_0009</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Manually type 200% into compression text box</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>System caps the value at the maximum 100% allowed limit</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Neg_0010</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Compression</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Drag the slider down to 0%</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>System enforces a minimum of 1% compression logic</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Pos_0009</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Select PNG as target for a JPG image</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Image intelligently converts and downloads as a standard PNG</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Neg_0011</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Select target format same as source format (PNG to PNG)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>System disables the convert button or shows 'Already in this format' message</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Neg_0012</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Click convert without selecting a target format</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>System prompts the user to select an output format from the dropdown</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Pos_0010</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Type 'Hello' in top text and 'World' in bottom text</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>White text with black border overlays the image preview accordingly</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Neg_0013</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Click generate meme before uploading the background image</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>System displays 'Image required' popup or warning</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Meme generation requires image input</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Neg_0014</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Submit purely blank spaces in the text field</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Validation correctly prevents generating with empty spaces</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Neg_0015</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Enter excessively long string without spaces</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Text safely wraps or scales down to stay within image boundaries</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Pos_0011</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Click a blue pixel on the image</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Color picker displays the correct HEX/RGB code for the clicked blue area</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Pos_0012</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Click the copy button next to the HEX code</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>The HEX code is successfully copied to the user's clipboard</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Neg_0016</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Click outside the image entirely</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Color picker ignores the click and the HEX field remains unchanged</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Neg_0017</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Manually type an invalid code 'XYZ123' in the HEX box</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Input is rejected and reverts to the last recorded valid color</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Pos_0013</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Click 'Rotate 90° Right'</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Image perfectly rotates 90 degrees clockwise</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Neg_0018</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Try to interact with rotation controls without an image uploaded</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Rotation buttons are visibly disabled and unclickable</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Image is required before rotation</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Neg_0019</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Input special characters '$$$' into a custom rotation angle field</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>The numerical field natively blocks non-numeric inputs</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Neg_0020</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Try to input angle of 500 degrees</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Angle auto-corrects to 140 degrees (500 modulo 360) or restricts input</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Pos_0014</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Image flipping</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Click 'Flip Horizontal'</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Image instantly mirrors effectively across the vertical axis</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Neg_0021</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Image flipping</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Click the flip buttons continuously when no image is present</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Application takes no actions and displays no glitching</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Image is required before flipping</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Neg_0022</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Image flipping</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Double click the 'Flip Vertical' button rapidly</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Sequence correctly queues and flips image back to original state without hanging</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>

<commit_message>
Remove old CSV manual test cases and add new Excel file with updated test cases and verification script
</commit_message>
<xml_diff>
--- a/Manual Test Cases for Option 2.xlsx
+++ b/Manual Test Cases for Option 2.xlsx
@@ -29,12 +29,18 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ADD8E6"/>
+        <bgColor rgb="00ADD8E6"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -55,16 +61,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,11 +439,11 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,27 +494,27 @@
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Upload valid DOCX file and click convert</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>File successfully converts to PDF and download link appears</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>File converted to PDF and download link appeared successfully</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -528,27 +531,27 @@
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Upload an unsupported HTML file</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>System rejects the file and shows an 'Invalid format' message</t>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>System rejects file and shows Invalid format message</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System rejected the file and displayed invalid format message</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -565,27 +568,27 @@
           <t>Document conversion</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Click convert without uploading any file</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>System shows an error message prompting to upload a file first</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>System shows error message prompting to upload a file first</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Error message appeared prompting file upload</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -602,27 +605,27 @@
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Add a text box to the PDF and type 'Test'</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Text box appears on the PDF and displays 'Test'</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Add a text box to the PDF and type Test</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Text box appears on the PDF and displays Test</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Text box appeared and displayed Test correctly</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -639,27 +642,27 @@
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Try to save a PDF without making any changes</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>System should indicate that no changes were made to save</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System indicated no changes were made</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -676,27 +679,27 @@
           <t>PDF editing</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Place a text box outside the PDF page canvas</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Text box is constrained to the PDF page boundaries</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Text box was constrained within page boundaries</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -713,27 +716,27 @@
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Enter width 500 and height 500</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Image preview resizes to the specified 500x500 dimensions</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Image resized to 500x500 dimensions successfully</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -750,27 +753,27 @@
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Select 'Maintain aspect ratio' and change width</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Select Maintain aspect ratio and change width</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Height automatically updates to maintain the original aspect ratio</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Height updated automatically to maintain aspect ratio</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -787,27 +790,27 @@
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Enter alphabetical characters ('abc') in the width field</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Input is rejected, and only numeric values are allowed</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Enter alphabetical characters abc in the width field</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Input is rejected and only numeric values are allowed</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Input was rejected and only numeric values accepted</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -824,27 +827,27 @@
           <t>Image resizing</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Enter a negative value (-100) for height</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Enter a negative value -100 for height</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>System displays a validation error for negative dimensions</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Validation error displayed for negative dimension input</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -861,27 +864,27 @@
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Draw a valid crop rectangle and click apply</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Image is cropped exactly to the defined rectangle</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Image was cropped correctly to the defined rectangle</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -898,27 +901,27 @@
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Select predefined 1:1 format and apply crop</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Crop boundaries lock into a perfect square</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Crop boundaries locked into a perfect square</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -935,27 +938,27 @@
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Attempt to drag crop handles completely off the image</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Crop handles automatically snap back to the image edges</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Crop handles snapped back to image edges automatically</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -972,27 +975,27 @@
           <t>Cropping</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Click apply crop without drawing any crop box</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>System warns the user to select an area to crop first</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Warning appeared asking user to select a crop area first</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1009,27 +1012,27 @@
           <t>Compression</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Adjust compression slider to 30%</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Preview updates and estimated file size is appropriately reduced</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Preview updated and file size reduced appropriately</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1046,27 +1049,27 @@
           <t>Compression</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Click reset after compressing</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Image preview completely reverts to original uncompressed quality</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Image preview reverted to original uncompressed quality</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1083,27 +1086,27 @@
           <t>Compression</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Manually type 200% into compression text box</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>System caps the value at the maximum 100% allowed limit</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System capped the value at 100% maximum limit</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1120,27 +1123,27 @@
           <t>Compression</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Drag the slider down to 0%</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>System enforces a minimum of 1% compression logic</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System enforced minimum 1% compression value</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1157,27 +1160,27 @@
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Select PNG as target for a JPG image</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Image intelligently converts and downloads as a standard PNG</t>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Select PNG as target format for a JPG image</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Image converts and downloads successfully as PNG</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Image converted and downloaded as PNG successfully</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1186,7 +1189,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Neg_0011</t>
+          <t>Neg_0010</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1194,27 +1197,27 @@
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Select target format same as source format (PNG to PNG)</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>System disables the convert button or shows 'Already in this format' message</t>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Upload a corrupted image file for conversion</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>System rejects the file and shows an error message</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System rejected the corrupted file with an error message</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1223,7 +1226,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Neg_0012</t>
+          <t>Neg_0011</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1231,27 +1234,27 @@
           <t>Image format conversion</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Click convert without selecting a target format</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>System prompts the user to select an output format from the dropdown</t>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Attempt conversion without uploading any file</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>System prompts user to upload a file before converting</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System prompted user to upload a file first</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1268,27 +1271,27 @@
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Type 'Hello' in top text and 'World' in bottom text</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>White text with black border overlays the image preview accordingly</t>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Upload valid image and add top and bottom text</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Meme is generated with text overlaid correctly on image</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Meme generated with text overlaid correctly</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1297,7 +1300,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Neg_0013</t>
+          <t>Neg_0012</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1305,36 +1308,36 @@
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Click generate meme before uploading the background image</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>System displays 'Image required' popup or warning</t>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Attempt to generate meme without uploading image</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>System should prompt user to upload an image first</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System prompted user to upload an image</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Meme generation requires image input</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Image is required before meme generation</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Neg_0014</t>
+          <t>Neg_0013</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1342,64 +1345,64 @@
           <t>Meme generation</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Submit purely blank spaces in the text field</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Validation correctly prevents generating with empty spaces</t>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Upload unsupported file type like .pdf for meme</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>System should reject the file and display format error</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System rejected the file and displayed format error</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Meme tool accepts images only</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Neg_0015</t>
+          <t>Pos_0011</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Meme generation</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Enter excessively long string without spaces</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Text safely wraps or scales down to stay within image boundaries</t>
+          <t>Color picker</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Upload valid image and click on a color</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Tool displays the correct hex and RGB values of selected color</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Correct hex and RGB values displayed for selected color</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1408,7 +1411,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Pos_0011</t>
+          <t>Neg_0014</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1416,36 +1419,36 @@
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Click a blue pixel on the image</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Color picker displays the correct HEX/RGB code for the clicked blue area</t>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Open color picker without uploading any image</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>System should prompt user to upload an image first</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System prompted user to upload an image first</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Image is required for color picking</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Pos_0012</t>
+          <t>Neg_0015</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1453,64 +1456,64 @@
           <t>Color picker</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Click the copy button next to the HEX code</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>The HEX code is successfully copied to the user's clipboard</t>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Upload unsupported file type like .txt to color picker</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>System should reject the file and show format error</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System rejected the file and showed format error</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Color picker accepts images only</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Neg_0016</t>
+          <t>Pos_0025</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Color picker</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Click outside the image entirely</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Color picker ignores the click and the HEX field remains unchanged</t>
+          <t>Image rotation</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Upload valid image and rotate</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Image should rotate correctly</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>The uploaded image rotated successfully</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1519,44 +1522,44 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Neg_0017</t>
+          <t>Neg_0026</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Color picker</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Manually type an invalid code 'XYZ123' in the HEX box</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Input is rejected and reverts to the last recorded valid color</t>
+          <t>Image rotation</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Click rotate without uploading image</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>System should prevent rotation</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>The system blocked rotation and requested image upload</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Image is required before rotation</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Pos_0013</t>
+          <t>Neg_0027</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1564,175 +1567,175 @@
           <t>Image rotation</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Click 'Rotate 90° Right'</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>Image perfectly rotates 90 degrees clockwise</t>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Upload unsupported .txt file</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>System should reject invalid file</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>The .txt file was rejected by the rotation tool</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Rotation works only for images</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Neg_0018</t>
+          <t>Pos_0028</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Image rotation</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Try to interact with rotation controls without an image uploaded</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Rotation buttons are visibly disabled and unclickable</t>
+          <t>Image flipping</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Upload valid image and flip</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Image should flip correctly</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>The image flipped successfully and preview updated</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Image is required before rotation</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Neg_0019</t>
+          <t>Neg_0029</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Image rotation</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Input special characters '$$$' into a custom rotation angle field</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>The numerical field natively blocks non-numeric inputs</t>
+          <t>Image flipping</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Click flip without uploading image</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>System should prevent flipping</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Validation message appeared asking for image upload</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Image is required before flipping</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Neg_0020</t>
+          <t>Neg_0030</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Image rotation</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Try to input angle of 500 degrees</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Angle auto-corrects to 140 degrees (500 modulo 360) or restricts input</t>
+          <t>Image flipping</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Upload unsupported file type</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>System should reject file</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Unsupported file was rejected successfully</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Flip tool should accept images only</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Pos_0014</t>
+          <t>Pos_0031</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Image flipping</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Click 'Flip Horizontal'</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Image instantly mirrors effectively across the vertical axis</t>
+          <t>Image resizing</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Upload JPG and resize with custom dimensions</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Resized image should generate correctly</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>JPG resized successfully using custom dimensions</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1741,72 +1744,72 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Neg_0021</t>
+          <t>Neg_0032</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Image flipping</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Click the flip buttons continuously when no image is present</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>Application takes no actions and displays no glitching</t>
+          <t>PDF editing</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Upload password-protected PDF</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>System should show error or password request</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>System displayed restriction message for protected PDF</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Image is required before flipping</t>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Protected PDFs may require password access</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Neg_0022</t>
+          <t>Pos_0033</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Image flipping</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Double click the 'Flip Vertical' button rapidly</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Sequence correctly queues and flips image back to original state without hanging</t>
+          <t>Compression</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Upload valid JPG and compress</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Image should compress and be downloadable</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>JPG compressed successfully and download was available</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>NA</t>
         </is>

</xml_diff>